<commit_message>
Marcar 37 atividades vencidas como CONCLUÍDO (100%)
A pedido do usuário, todas as atividades com prazo anterior a hoje (22/06/2026)
que estavam PENDENTE/EM ANDAMENTO foram marcadas como CONCLUÍDO e % Conclusão
ajustado para 100%. Resultado: 99 CONCLUÍDO, 43 PENDENTE, 1 EM ANDAMENTO,
0 vencidos em aberto.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaQa9GJrUwmBhw6Gk2YbRh
</commit_message>
<xml_diff>
--- a/NEC_Eventos_Reestruturado_v4.xlsx
+++ b/NEC_Eventos_Reestruturado_v4.xlsx
@@ -13465,11 +13465,11 @@
         <v>46186</v>
       </c>
       <c r="G34" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I34" s="76" t="n"/>
@@ -13750,11 +13750,11 @@
         <v>46191</v>
       </c>
       <c r="G43" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I43" s="77" t="n"/>
@@ -14000,11 +14000,11 @@
         <v>46191</v>
       </c>
       <c r="G51" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I51" s="77" t="n"/>
@@ -14095,11 +14095,11 @@
         <v>46168</v>
       </c>
       <c r="G54" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I54" s="76" t="n"/>
@@ -14252,11 +14252,11 @@
         <v>46153</v>
       </c>
       <c r="G59" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I59" s="77" t="n"/>
@@ -14285,11 +14285,11 @@
         <v>46184</v>
       </c>
       <c r="G60" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I60" s="76" t="n"/>
@@ -14503,11 +14503,11 @@
         <v>46125</v>
       </c>
       <c r="G68" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H68" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I68" s="76" t="n"/>
@@ -14536,11 +14536,11 @@
         <v>46140</v>
       </c>
       <c r="G69" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H69" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I69" s="77" t="n"/>
@@ -14569,11 +14569,11 @@
         <v>46185</v>
       </c>
       <c r="G70" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H70" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I70" s="76" t="n"/>
@@ -14602,11 +14602,11 @@
         <v>46155</v>
       </c>
       <c r="G71" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I71" s="77" t="n"/>
@@ -14635,11 +14635,11 @@
         <v>46194</v>
       </c>
       <c r="G72" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I72" s="76" t="n"/>
@@ -14668,11 +14668,11 @@
         <v>46185</v>
       </c>
       <c r="G73" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I73" s="77" t="n"/>
@@ -14701,11 +14701,11 @@
         <v>46194</v>
       </c>
       <c r="G74" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I74" s="76" t="n"/>
@@ -14734,11 +14734,11 @@
         <v>46170</v>
       </c>
       <c r="G75" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H75" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I75" s="77" t="n"/>
@@ -14829,11 +14829,11 @@
         <v>46155</v>
       </c>
       <c r="G78" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I78" s="76" t="n"/>
@@ -14858,11 +14858,11 @@
         <v>46155</v>
       </c>
       <c r="G79" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I79" s="77" t="inlineStr">
@@ -14891,11 +14891,11 @@
         <v>46194</v>
       </c>
       <c r="G80" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I80" s="76" t="inlineStr">
@@ -14924,11 +14924,11 @@
         <v>46194</v>
       </c>
       <c r="G81" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I81" s="77" t="inlineStr">
@@ -14957,11 +14957,11 @@
         <v>46194</v>
       </c>
       <c r="G82" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I82" s="76" t="inlineStr">
@@ -14990,11 +14990,11 @@
         <v>46155</v>
       </c>
       <c r="G83" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I83" s="77" t="inlineStr">
@@ -15023,11 +15023,11 @@
         <v>46194</v>
       </c>
       <c r="G84" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I84" s="76" t="inlineStr">
@@ -15056,11 +15056,11 @@
         <v>46194</v>
       </c>
       <c r="G85" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H85" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I85" s="77" t="inlineStr">
@@ -15089,11 +15089,11 @@
         <v>46194</v>
       </c>
       <c r="G86" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I86" s="76" t="inlineStr">
@@ -15122,11 +15122,11 @@
         <v>46194</v>
       </c>
       <c r="G87" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H87" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I87" s="77" t="inlineStr">
@@ -15155,11 +15155,11 @@
         <v>46194</v>
       </c>
       <c r="G88" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I88" s="76" t="inlineStr">
@@ -15188,11 +15188,11 @@
         <v>46194</v>
       </c>
       <c r="G89" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H89" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I89" s="77" t="inlineStr">
@@ -15221,11 +15221,11 @@
         <v>46194</v>
       </c>
       <c r="G90" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H90" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I90" s="76" t="inlineStr">
@@ -15254,11 +15254,11 @@
         <v>46194</v>
       </c>
       <c r="G91" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I91" s="77" t="inlineStr">
@@ -15287,11 +15287,11 @@
         <v>46155</v>
       </c>
       <c r="G92" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I92" s="76" t="inlineStr">
@@ -15353,11 +15353,11 @@
         <v>46194</v>
       </c>
       <c r="G94" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H94" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I94" s="76" t="inlineStr">
@@ -15387,11 +15387,11 @@
         <v>46194</v>
       </c>
       <c r="G95" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I95" s="77" t="n"/>
@@ -15651,11 +15651,11 @@
         <v>46174</v>
       </c>
       <c r="G103" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H103" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I103" s="77" t="n"/>
@@ -15748,11 +15748,11 @@
         <v>46164</v>
       </c>
       <c r="G106" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I106" s="76" t="n"/>
@@ -15812,11 +15812,11 @@
         <v>46194</v>
       </c>
       <c r="G108" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I108" s="76" t="n"/>
@@ -15878,11 +15878,11 @@
         <v>46194</v>
       </c>
       <c r="G110" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H110" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I110" s="76" t="n"/>
@@ -15915,11 +15915,11 @@
         <v>46185</v>
       </c>
       <c r="G111" s="20" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H111" s="14" t="inlineStr">
         <is>
-          <t>EM ANDAMENTO</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I111" s="77" t="n"/>
@@ -15952,11 +15952,11 @@
         <v>46185</v>
       </c>
       <c r="G112" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="I112" s="76" t="n"/>

</xml_diff>

<commit_message>
Corrigir corrupção que disparava aviso de recuperação do Excel
Causa: validação de dados em DB_ATIVIDADES tinha formula1 inválida
(_xlfn._LONGTEXT com 462 chars > limite de 255), resíduo das edições do
usuário no Excel ao ter uma lista de dropdown longa demais. O Excel não
conseguia ler e pedia recuperação ao abrir.

Fix: removidas todas as validações da aba e reconstruídas 3 limpas:
- Status (H): lista CONCLUÍDO,EM ANDAMENTO,PENDENTE,ATRASADO,-
- Responsável (E): lista com os 5 responsáveis reais (57 chars)
- Prazo (F): validação de data

Varredura confirmou: era o único problema; tabelas e nomes definidos
sem duplicação, contagens de CF e validações consistentes.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaQa9GJrUwmBhw6Gk2YbRh
</commit_message>
<xml_diff>
--- a/NEC_Eventos_Reestruturado_v4.xlsx
+++ b/NEC_Eventos_Reestruturado_v4.xlsx
@@ -17214,13 +17214,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="D4:D146 E4:E21 E25:E62 E68:E146 I79:I94" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" promptTitle="Responsável" type="list">
-      <formula1>_xlfn._LONGTEXT("1 lâmina - Propaganda ou similar, de produção própria, aprovada pelo CONASEMS,10 unidades,130000,24m²,30 segundos - Em looping no painel de LED,4 unidades,500,00*,6 unidades,Ação promocional - No próprio Estande (se houver),Briefing,Briefing para agênci,C","ontrato (cota),Contrato Palestrantes,Contratos Palestrantes,Coordenador,Documentação Prefeitura (RJ/Gramado),Documentação Prefeitura (SP/RJ/Gramado),EM Aprovada,EM COTA,EM COTA Aprovada")</formula1>
-    </dataValidation>
-    <dataValidation sqref="H4:H146" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" promptTitle="Status" type="list">
+    <dataValidation sqref="H4:H146" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Status" type="list">
       <formula1>"CONCLUÍDO,EM ANDAMENTO,PENDENTE,ATRASADO,-"</formula1>
     </dataValidation>
-    <dataValidation sqref="F4:F146" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data inválida" error="Insira uma data válida (DD/MM/AAAA) ou deixe em branco. Texto não é permitido nesta coluna." promptTitle="Prazo da Atividade" prompt="Insira a data no formato DD/MM/AAAA.&#10;Deixe em branco se ainda não houver prazo definido." type="date" operator="greaterThanOrEqual">
+    <dataValidation sqref="E4:E146" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Responsável" type="list">
+      <formula1>"Eventos,Fernando Azato,Janaina Silva,Marcio,Time de Marca"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F4:F146" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Data inválida" error="Insira uma data válida (DD/MM/AAAA) ou deixe em branco." promptTitle="Prazo da Atividade" prompt="Insira a data no formato DD/MM/AAAA. Deixe em branco se não houver prazo." type="date" operator="greaterThanOrEqual">
       <formula1>43831</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>